<commit_message>
Catálogo: layout padrão Role|Level|Location|Cost/h|Rate/h para todos os clientes, inclusive JnJ
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bdbu36GthA9GDEUe8SjfAs
</commit_message>
<xml_diff>
--- a/Perfis_e_Taxas.xlsx
+++ b/Perfis_e_Taxas.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="33">
   <si>
     <t>Role</t>
   </si>
@@ -69,17 +69,6 @@
     <t>Data Visualization Analyst</t>
   </si>
   <si>
-    <t>Roles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experience level
-(See instructions tab for experience level definitions)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TCS without
-taxes 2026 BRL</t>
-  </si>
-  <si>
     <t>Developer: SAP BASIS</t>
   </si>
   <si>
@@ -116,7 +105,7 @@
     <t>Catálogo de perfis e taxas — uma aba por cliente</t>
   </si>
   <si>
-    <t>A aba JnJ vem do arquivo do cliente (amostra): substitua pelos dados oficiais mantendo o cabeçalho (Roles, Experience level, taxa sem impostos).</t>
+    <t>Layout padrão de todos os clientes: Role | Level | Location | Cost/h | Rate/h. Os valores da JnJ são uma amostra (Rate/h em BRL, sem impostos): substitua pelos oficiais.</t>
   </si>
   <si>
     <t>Cada aba nova (cliente) é criada pelo app a partir de outra aba ou em branco; o app lê as colunas pelo cabeçalho.</t>
@@ -129,9 +118,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;R$&quot; #,##0.00"/>
-  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
@@ -148,7 +134,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -158,16 +144,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E5F3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFB4C7E7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8CBAD"/>
       </patternFill>
     </fill>
   </fills>
@@ -183,18 +159,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="4" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -696,235 +665,264 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="44" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="5" width="12" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B2" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D2" s="1"/>
+      <c r="E2" s="1">
+        <v>142.91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="D3" s="1"/>
+      <c r="E3" s="1">
+        <v>178.08</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>21</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="6">
-        <v>142.91</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="D4" s="1"/>
+      <c r="E4" s="1">
+        <v>109.93</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>21</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1">
+        <v>167.09</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1">
+        <v>198.97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="6">
-        <v>178.08</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>24</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="6">
-        <v>109.93</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="6">
-        <v>167.09</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="6">
-        <v>198.97</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>26</v>
       </c>
-      <c r="B7" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="6"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>26</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B17" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="6"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>26</v>
       </c>
-      <c r="B9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="6"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B18" t="s">
+        <v>19</v>
+      </c>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>27</v>
       </c>
-      <c r="B10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="6"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="B19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>27</v>
       </c>
-      <c r="B11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="6"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="B20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>27</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="6"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" s="6"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="6"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" t="s">
-        <v>22</v>
-      </c>
-      <c r="C15" s="6"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="6"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="6"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>29</v>
-      </c>
-      <c r="B18" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" s="6"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" t="s">
-        <v>23</v>
-      </c>
-      <c r="C19" s="6"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>30</v>
-      </c>
-      <c r="B20" t="s">
-        <v>25</v>
-      </c>
-      <c r="C20" s="6"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>30</v>
-      </c>
-      <c r="B21" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="6"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>31</v>
-      </c>
-      <c r="B22" t="s">
-        <v>23</v>
-      </c>
-      <c r="C22" s="6"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>31</v>
-      </c>
-      <c r="B23" t="s">
-        <v>25</v>
-      </c>
-      <c r="C23" s="6"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C1"/>
+  <autoFilter ref="A1:E1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -938,24 +936,24 @@
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>32</v>
+    <row r="1" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrige cor dos entregáveis e usa layout padrão no catálogo (inclusive JnJ) (#5)
* Corrige cor do nome dos entregáveis na timeline (texto branco ilegível)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bdbu36GthA9GDEUe8SjfAs

* Catálogo: layout padrão Role|Level|Location|Cost/h|Rate/h para todos os clientes, inclusive JnJ

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bdbu36GthA9GDEUe8SjfAs

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Perfis_e_Taxas.xlsx
+++ b/Perfis_e_Taxas.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="33">
   <si>
     <t>Role</t>
   </si>
@@ -69,17 +69,6 @@
     <t>Data Visualization Analyst</t>
   </si>
   <si>
-    <t>Roles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experience level
-(See instructions tab for experience level definitions)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TCS without
-taxes 2026 BRL</t>
-  </si>
-  <si>
     <t>Developer: SAP BASIS</t>
   </si>
   <si>
@@ -116,7 +105,7 @@
     <t>Catálogo de perfis e taxas — uma aba por cliente</t>
   </si>
   <si>
-    <t>A aba JnJ vem do arquivo do cliente (amostra): substitua pelos dados oficiais mantendo o cabeçalho (Roles, Experience level, taxa sem impostos).</t>
+    <t>Layout padrão de todos os clientes: Role | Level | Location | Cost/h | Rate/h. Os valores da JnJ são uma amostra (Rate/h em BRL, sem impostos): substitua pelos oficiais.</t>
   </si>
   <si>
     <t>Cada aba nova (cliente) é criada pelo app a partir de outra aba ou em branco; o app lê as colunas pelo cabeçalho.</t>
@@ -129,9 +118,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;R$&quot; #,##0.00"/>
-  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
@@ -148,7 +134,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -158,16 +144,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E5F3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFB4C7E7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8CBAD"/>
       </patternFill>
     </fill>
   </fills>
@@ -183,18 +159,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="4" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -696,235 +665,264 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="44" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="5" width="12" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B2" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D2" s="1"/>
+      <c r="E2" s="1">
+        <v>142.91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="D3" s="1"/>
+      <c r="E3" s="1">
+        <v>178.08</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>21</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="6">
-        <v>142.91</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="D4" s="1"/>
+      <c r="E4" s="1">
+        <v>109.93</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>21</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1">
+        <v>167.09</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1">
+        <v>198.97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="6">
-        <v>178.08</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>24</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="6">
-        <v>109.93</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="6">
-        <v>167.09</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="6">
-        <v>198.97</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>26</v>
       </c>
-      <c r="B7" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="6"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>26</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B17" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="6"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>26</v>
       </c>
-      <c r="B9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="6"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B18" t="s">
+        <v>19</v>
+      </c>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>27</v>
       </c>
-      <c r="B10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="6"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="B19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>27</v>
       </c>
-      <c r="B11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="6"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="B20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>27</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="6"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" s="6"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="6"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" t="s">
-        <v>22</v>
-      </c>
-      <c r="C15" s="6"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="6"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="6"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>29</v>
-      </c>
-      <c r="B18" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" s="6"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" t="s">
-        <v>23</v>
-      </c>
-      <c r="C19" s="6"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>30</v>
-      </c>
-      <c r="B20" t="s">
-        <v>25</v>
-      </c>
-      <c r="C20" s="6"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>30</v>
-      </c>
-      <c r="B21" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="6"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>31</v>
-      </c>
-      <c r="B22" t="s">
-        <v>23</v>
-      </c>
-      <c r="C22" s="6"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>31</v>
-      </c>
-      <c r="B23" t="s">
-        <v>25</v>
-      </c>
-      <c r="C23" s="6"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C1"/>
+  <autoFilter ref="A1:E1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -938,24 +936,24 @@
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>32</v>
+    <row r="1" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Painel de margens GM/GPM, racional ao passar o mouse, salário sugerido e Rate net/h padrão
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bdbu36GthA9GDEUe8SjfAs
</commit_message>
<xml_diff>
--- a/Perfis_e_Taxas.xlsx
+++ b/Perfis_e_Taxas.xlsx
@@ -27,7 +27,7 @@
     <t>Cost/h</t>
   </si>
   <si>
-    <t>Rate/h</t>
+    <t>Rate net/h</t>
   </si>
   <si>
     <t>Notes</t>
@@ -105,7 +105,7 @@
     <t>Catálogo de perfis e taxas — uma aba por cliente</t>
   </si>
   <si>
-    <t>Layout padrão de todos os clientes: Role | Level | Location | Cost/h | Rate/h. Os valores da JnJ são uma amostra (Rate/h em BRL, sem impostos): substitua pelos oficiais.</t>
+    <t>Layout padrão de todos os clientes: Role | Level | Location | Cost/h | Rate net/h. Os valores da JnJ são uma amostra (Rate net/h em BRL, sem impostos): substitua pelos oficiais.</t>
   </si>
   <si>
     <t>Cada aba nova (cliente) é criada pelo app a partir de outra aba ou em branco; o app lê as colunas pelo cabeçalho.</t>

</xml_diff>

<commit_message>
Painel de margens GM/GPM, racional ao passar o mouse, salário sugerido e Rate net/h padrão (#6)
Claude-Session: https://claude.ai/code/session_01Bdbu36GthA9GDEUe8SjfAs

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Perfis_e_Taxas.xlsx
+++ b/Perfis_e_Taxas.xlsx
@@ -27,7 +27,7 @@
     <t>Cost/h</t>
   </si>
   <si>
-    <t>Rate/h</t>
+    <t>Rate net/h</t>
   </si>
   <si>
     <t>Notes</t>
@@ -105,7 +105,7 @@
     <t>Catálogo de perfis e taxas — uma aba por cliente</t>
   </si>
   <si>
-    <t>Layout padrão de todos os clientes: Role | Level | Location | Cost/h | Rate/h. Os valores da JnJ são uma amostra (Rate/h em BRL, sem impostos): substitua pelos oficiais.</t>
+    <t>Layout padrão de todos os clientes: Role | Level | Location | Cost/h | Rate net/h. Os valores da JnJ são uma amostra (Rate net/h em BRL, sem impostos): substitua pelos oficiais.</t>
   </si>
   <si>
     <t>Cada aba nova (cliente) é criada pelo app a partir de outra aba ou em branco; o app lê as colunas pelo cabeçalho.</t>

</xml_diff>